<commit_message>
Add full citations for the reference single-cell datasets
Four of the six published datasets had no publication listed in the README, and
the spreadsheet carried author-year stubs only. Each now has the full title,
journal, volume/pages and DOI, verified against the PubMed record linked from
its GEO accession. Accessions link to GEO.

Also records that GSE114374 (Kinchen) is a mixed-species series and only the
mouse samples are used, confirmed from the object's gene symbols.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dataset_Documentation.xlsx
+++ b/Dataset_Documentation.xlsx
@@ -667,7 +667,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Degirmenci et al., Nature 2018</t>
+          <t>Degirmenci B, Valenta T, Dimitrieva S, Hausmann G, Basler K. GLI1-expressing mesenchymal cells form the essential Wnt-secreting niche for colon stem cells. Nature 2018;558(7710):449-453. doi:10.1038/s41586-018-0190-3</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Kinchen et al., Cell 2018</t>
+          <t>Kinchen J, Chen HH, Parikh K, et al. Structural remodeling of the human colonic mesenchyme in inflammatory bowel disease. Cell 2018;175(2):372-386.e17. doi:10.1016/j.cell.2018.08.067</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>3 healthy-control samples combined in one matrix; immune cells removed via Ptprc.</t>
+          <t>3 healthy-control samples combined in one matrix; immune cells removed via Ptprc. NOTE: GSE114374 is a mixed-species series (human + mouse); only the mouse samples are used here.</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>McCarthy et al., Cell Stem Cell 2020</t>
+          <t>McCarthy N, Manieri E, Storm EE, et al. Distinct mesenchymal cell populations generate the essential intestinal BMP signaling gradient. Cell Stem Cell 2020;26(3):391-402.e5. doi:10.1016/j.stem.2020.01.008</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Roulis et al., Nature 2020</t>
+          <t>Roulis M, Kaklamanos A, Schernthanner M, et al. Paracrine orchestration of intestinal tumorigenesis by a mesenchymal niche. Nature 2020;580(7804):524-529. doi:10.1038/s41586-020-2166-3</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">

</xml_diff>